<commit_message>
Tweaks to exposure parameter file.
</commit_message>
<xml_diff>
--- a/Inputs/PFOA_template_parameters_Exposure.xlsx
+++ b/Inputs/PFOA_template_parameters_Exposure.xlsx
@@ -6748,8 +6748,8 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1022ded5d06c8e179fc5cb1f37040178">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="edea5721ce64dde47a72ba01132ba27b" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
     <xsd:import namespace="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint.v3"/>
@@ -7282,26 +7282,7 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5B6850C-32F9-4402-840F-018327152438}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
-    <ds:schemaRef ds:uri="41d9f072-86bf-4c63-b117-debf50ff4701"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{914A4456-185A-48CA-AFCB-6875271AD8E5}"/>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>